<commit_message>
xong owd cơ bản
</commit_message>
<xml_diff>
--- a/CCS.xlsx
+++ b/CCS.xlsx
@@ -2086,7 +2086,10 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2095,32 +2098,17 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2128,14 +2116,26 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3837,7 +3837,7 @@
       <c r="R5" s="14"/>
     </row>
     <row r="6" spans="1:27" ht="150" customHeight="1">
-      <c r="A6" s="50" t="s">
+      <c r="A6" s="60" t="s">
         <v>30</v>
       </c>
       <c r="B6" s="16" t="s">
@@ -3890,7 +3890,7 @@
       <c r="AA6" s="23"/>
     </row>
     <row r="7" spans="1:27" ht="150" customHeight="1">
-      <c r="A7" s="51"/>
+      <c r="A7" s="52"/>
       <c r="B7" s="18" t="s">
         <v>37</v>
       </c>
@@ -3939,7 +3939,7 @@
       <c r="AA7" s="25"/>
     </row>
     <row r="8" spans="1:27" ht="150" customHeight="1">
-      <c r="A8" s="51"/>
+      <c r="A8" s="52"/>
       <c r="B8" s="18" t="s">
         <v>42</v>
       </c>
@@ -3990,16 +3990,16 @@
       <c r="AA8" s="25"/>
     </row>
     <row r="9" spans="1:27" ht="150" customHeight="1">
-      <c r="A9" s="54" t="s">
+      <c r="A9" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="53" t="s">
+      <c r="B9" s="61" t="s">
         <v>47</v>
       </c>
       <c r="C9" s="19">
         <v>1</v>
       </c>
-      <c r="D9" s="50" t="s">
+      <c r="D9" s="60" t="s">
         <v>48</v>
       </c>
       <c r="E9" s="26" t="s">
@@ -4043,12 +4043,12 @@
       <c r="AA9" s="25"/>
     </row>
     <row r="10" spans="1:27" ht="150" customHeight="1">
-      <c r="A10" s="51"/>
-      <c r="B10" s="51"/>
+      <c r="A10" s="52"/>
+      <c r="B10" s="52"/>
       <c r="C10" s="19">
         <v>2</v>
       </c>
-      <c r="D10" s="51"/>
+      <c r="D10" s="52"/>
       <c r="E10" s="26" t="s">
         <v>53</v>
       </c>
@@ -4090,12 +4090,12 @@
       <c r="AA10" s="25"/>
     </row>
     <row r="11" spans="1:27" ht="150" customHeight="1">
-      <c r="A11" s="51"/>
-      <c r="B11" s="51"/>
+      <c r="A11" s="52"/>
+      <c r="B11" s="52"/>
       <c r="C11" s="19">
         <v>3</v>
       </c>
-      <c r="D11" s="52"/>
+      <c r="D11" s="53"/>
       <c r="E11" s="44" t="s">
         <v>56</v>
       </c>
@@ -4135,12 +4135,12 @@
       <c r="AA11" s="25"/>
     </row>
     <row r="12" spans="1:27" ht="150" customHeight="1">
-      <c r="A12" s="51"/>
-      <c r="B12" s="51"/>
+      <c r="A12" s="52"/>
+      <c r="B12" s="52"/>
       <c r="C12" s="9">
         <v>4</v>
       </c>
-      <c r="D12" s="55" t="s">
+      <c r="D12" s="51" t="s">
         <v>59</v>
       </c>
       <c r="E12" s="10" t="s">
@@ -4182,12 +4182,12 @@
       <c r="AA12" s="25"/>
     </row>
     <row r="13" spans="1:27" ht="150" customHeight="1">
-      <c r="A13" s="51"/>
-      <c r="B13" s="51"/>
+      <c r="A13" s="52"/>
+      <c r="B13" s="52"/>
       <c r="C13" s="9">
         <v>5</v>
       </c>
-      <c r="D13" s="51"/>
+      <c r="D13" s="52"/>
       <c r="E13" s="10" t="s">
         <v>53</v>
       </c>
@@ -4227,12 +4227,12 @@
       <c r="AA13" s="25"/>
     </row>
     <row r="14" spans="1:27" ht="150" customHeight="1">
-      <c r="A14" s="52"/>
-      <c r="B14" s="52"/>
+      <c r="A14" s="53"/>
+      <c r="B14" s="53"/>
       <c r="C14" s="9">
         <v>6</v>
       </c>
-      <c r="D14" s="52"/>
+      <c r="D14" s="53"/>
       <c r="E14" s="45" t="s">
         <v>56</v>
       </c>
@@ -4272,19 +4272,19 @@
       <c r="AA14" s="25"/>
     </row>
     <row r="15" spans="1:27" ht="150" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="60" t="s">
         <v>62</v>
       </c>
-      <c r="B15" s="53" t="s">
+      <c r="B15" s="61" t="s">
         <v>63</v>
       </c>
       <c r="C15" s="9">
         <v>1</v>
       </c>
-      <c r="D15" s="50" t="s">
+      <c r="D15" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="E15" s="56" t="s">
+      <c r="E15" s="63" t="s">
         <v>65</v>
       </c>
       <c r="F15" s="18" t="s">
@@ -4329,17 +4329,17 @@
       <c r="AA15" s="25"/>
     </row>
     <row r="16" spans="1:27" ht="150" customHeight="1">
-      <c r="A16" s="51"/>
-      <c r="B16" s="51"/>
+      <c r="A16" s="52"/>
+      <c r="B16" s="52"/>
       <c r="C16" s="9">
         <v>2</v>
       </c>
-      <c r="D16" s="51"/>
-      <c r="E16" s="51"/>
-      <c r="F16" s="53" t="s">
+      <c r="D16" s="52"/>
+      <c r="E16" s="52"/>
+      <c r="F16" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="G16" s="53" t="s">
+      <c r="G16" s="61" t="s">
         <v>23</v>
       </c>
       <c r="H16" s="26" t="s">
@@ -4378,15 +4378,15 @@
       <c r="AA16" s="25"/>
     </row>
     <row r="17" spans="1:27" ht="150" customHeight="1">
-      <c r="A17" s="51"/>
-      <c r="B17" s="51"/>
+      <c r="A17" s="52"/>
+      <c r="B17" s="52"/>
       <c r="C17" s="9">
         <v>3</v>
       </c>
-      <c r="D17" s="51"/>
-      <c r="E17" s="52"/>
-      <c r="F17" s="52"/>
-      <c r="G17" s="52"/>
+      <c r="D17" s="52"/>
+      <c r="E17" s="53"/>
+      <c r="F17" s="53"/>
+      <c r="G17" s="53"/>
       <c r="H17" s="17" t="s">
         <v>71</v>
       </c>
@@ -4423,22 +4423,22 @@
       <c r="AA17" s="25"/>
     </row>
     <row r="18" spans="1:27" ht="150" customHeight="1">
-      <c r="A18" s="51"/>
-      <c r="B18" s="51"/>
+      <c r="A18" s="52"/>
+      <c r="B18" s="52"/>
       <c r="C18" s="9">
         <v>4</v>
       </c>
-      <c r="D18" s="51"/>
-      <c r="E18" s="56" t="s">
+      <c r="D18" s="52"/>
+      <c r="E18" s="63" t="s">
         <v>73</v>
       </c>
-      <c r="F18" s="53" t="s">
+      <c r="F18" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="G18" s="53" t="s">
+      <c r="G18" s="61" t="s">
         <v>23</v>
       </c>
-      <c r="H18" s="50" t="s">
+      <c r="H18" s="60" t="s">
         <v>74</v>
       </c>
       <c r="I18" s="17" t="s">
@@ -4470,16 +4470,16 @@
       <c r="AA18" s="24"/>
     </row>
     <row r="19" spans="1:27" ht="150" customHeight="1">
-      <c r="A19" s="51"/>
-      <c r="B19" s="51"/>
+      <c r="A19" s="52"/>
+      <c r="B19" s="52"/>
       <c r="C19" s="9">
         <v>5</v>
       </c>
-      <c r="D19" s="51"/>
-      <c r="E19" s="52"/>
-      <c r="F19" s="52"/>
-      <c r="G19" s="52"/>
-      <c r="H19" s="52"/>
+      <c r="D19" s="52"/>
+      <c r="E19" s="53"/>
+      <c r="F19" s="53"/>
+      <c r="G19" s="53"/>
+      <c r="H19" s="53"/>
       <c r="I19" s="17" t="s">
         <v>76</v>
       </c>
@@ -4509,12 +4509,12 @@
       <c r="AA19" s="24"/>
     </row>
     <row r="20" spans="1:27" ht="150" customHeight="1">
-      <c r="A20" s="51"/>
-      <c r="B20" s="51"/>
+      <c r="A20" s="52"/>
+      <c r="B20" s="52"/>
       <c r="C20" s="9">
         <v>6</v>
       </c>
-      <c r="D20" s="51"/>
+      <c r="D20" s="52"/>
       <c r="E20" s="26" t="s">
         <v>77</v>
       </c>
@@ -4556,12 +4556,12 @@
       <c r="AA20" s="24"/>
     </row>
     <row r="21" spans="1:27" ht="150" customHeight="1">
-      <c r="A21" s="51"/>
-      <c r="B21" s="51"/>
+      <c r="A21" s="52"/>
+      <c r="B21" s="52"/>
       <c r="C21" s="9">
         <v>7</v>
       </c>
-      <c r="D21" s="51"/>
+      <c r="D21" s="52"/>
       <c r="E21" s="26" t="s">
         <v>80</v>
       </c>
@@ -4603,13 +4603,13 @@
       <c r="AA21" s="24"/>
     </row>
     <row r="22" spans="1:27" ht="150" customHeight="1">
-      <c r="A22" s="51"/>
-      <c r="B22" s="51"/>
+      <c r="A22" s="52"/>
+      <c r="B22" s="52"/>
       <c r="C22" s="9">
         <v>8</v>
       </c>
-      <c r="D22" s="51"/>
-      <c r="E22" s="56" t="s">
+      <c r="D22" s="52"/>
+      <c r="E22" s="63" t="s">
         <v>83</v>
       </c>
       <c r="F22" s="18" t="s">
@@ -4650,13 +4650,13 @@
       <c r="AA22" s="24"/>
     </row>
     <row r="23" spans="1:27" ht="150" customHeight="1">
-      <c r="A23" s="51"/>
-      <c r="B23" s="51"/>
+      <c r="A23" s="52"/>
+      <c r="B23" s="52"/>
       <c r="C23" s="9">
         <v>9</v>
       </c>
-      <c r="D23" s="51"/>
-      <c r="E23" s="52"/>
+      <c r="D23" s="52"/>
+      <c r="E23" s="53"/>
       <c r="F23" s="18" t="s">
         <v>22</v>
       </c>
@@ -4695,19 +4695,19 @@
       <c r="AA23" s="24"/>
     </row>
     <row r="24" spans="1:27" ht="150" customHeight="1">
-      <c r="A24" s="51"/>
-      <c r="B24" s="51"/>
+      <c r="A24" s="52"/>
+      <c r="B24" s="52"/>
       <c r="C24" s="9">
         <v>10</v>
       </c>
-      <c r="D24" s="51"/>
-      <c r="E24" s="56" t="s">
+      <c r="D24" s="52"/>
+      <c r="E24" s="63" t="s">
         <v>87</v>
       </c>
-      <c r="F24" s="53" t="s">
+      <c r="F24" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="G24" s="53" t="s">
+      <c r="G24" s="61" t="s">
         <v>66</v>
       </c>
       <c r="H24" s="17" t="s">
@@ -4742,15 +4742,15 @@
       <c r="AA24" s="24"/>
     </row>
     <row r="25" spans="1:27" ht="150" customHeight="1">
-      <c r="A25" s="51"/>
-      <c r="B25" s="51"/>
+      <c r="A25" s="52"/>
+      <c r="B25" s="52"/>
       <c r="C25" s="9">
         <v>11</v>
       </c>
-      <c r="D25" s="51"/>
-      <c r="E25" s="51"/>
-      <c r="F25" s="51"/>
-      <c r="G25" s="51"/>
+      <c r="D25" s="52"/>
+      <c r="E25" s="52"/>
+      <c r="F25" s="52"/>
+      <c r="G25" s="52"/>
       <c r="H25" s="17" t="s">
         <v>90</v>
       </c>
@@ -4783,15 +4783,15 @@
       <c r="AA25" s="24"/>
     </row>
     <row r="26" spans="1:27" ht="150" customHeight="1">
-      <c r="A26" s="51"/>
-      <c r="B26" s="51"/>
+      <c r="A26" s="52"/>
+      <c r="B26" s="52"/>
       <c r="C26" s="9">
         <v>12</v>
       </c>
-      <c r="D26" s="51"/>
-      <c r="E26" s="51"/>
-      <c r="F26" s="51"/>
-      <c r="G26" s="51"/>
+      <c r="D26" s="52"/>
+      <c r="E26" s="52"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="52"/>
       <c r="H26" s="17" t="s">
         <v>92</v>
       </c>
@@ -4824,15 +4824,15 @@
       <c r="AA26" s="24"/>
     </row>
     <row r="27" spans="1:27" ht="150" customHeight="1">
-      <c r="A27" s="51"/>
-      <c r="B27" s="51"/>
+      <c r="A27" s="52"/>
+      <c r="B27" s="52"/>
       <c r="C27" s="9">
         <v>13</v>
       </c>
-      <c r="D27" s="51"/>
-      <c r="E27" s="51"/>
-      <c r="F27" s="51"/>
-      <c r="G27" s="51"/>
+      <c r="D27" s="52"/>
+      <c r="E27" s="52"/>
+      <c r="F27" s="52"/>
+      <c r="G27" s="52"/>
       <c r="H27" s="17" t="s">
         <v>93</v>
       </c>
@@ -4865,15 +4865,15 @@
       <c r="AA27" s="24"/>
     </row>
     <row r="28" spans="1:27" ht="150" customHeight="1">
-      <c r="A28" s="51"/>
-      <c r="B28" s="51"/>
+      <c r="A28" s="52"/>
+      <c r="B28" s="52"/>
       <c r="C28" s="9">
         <v>14</v>
       </c>
-      <c r="D28" s="51"/>
-      <c r="E28" s="52"/>
-      <c r="F28" s="52"/>
-      <c r="G28" s="52"/>
+      <c r="D28" s="52"/>
+      <c r="E28" s="53"/>
+      <c r="F28" s="53"/>
+      <c r="G28" s="53"/>
       <c r="H28" s="17" t="s">
         <v>94</v>
       </c>
@@ -4906,22 +4906,22 @@
       <c r="AA28" s="24"/>
     </row>
     <row r="29" spans="1:27" ht="150" customHeight="1">
-      <c r="A29" s="51"/>
-      <c r="B29" s="51"/>
+      <c r="A29" s="52"/>
+      <c r="B29" s="52"/>
       <c r="C29" s="9">
         <v>15</v>
       </c>
-      <c r="D29" s="51"/>
-      <c r="E29" s="50" t="s">
+      <c r="D29" s="52"/>
+      <c r="E29" s="60" t="s">
         <v>95</v>
       </c>
-      <c r="F29" s="53" t="s">
+      <c r="F29" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="G29" s="53" t="s">
+      <c r="G29" s="61" t="s">
         <v>96</v>
       </c>
-      <c r="H29" s="50" t="s">
+      <c r="H29" s="60" t="s">
         <v>97</v>
       </c>
       <c r="I29" s="17" t="s">
@@ -4953,16 +4953,16 @@
       <c r="AA29" s="24"/>
     </row>
     <row r="30" spans="1:27" ht="150" customHeight="1">
-      <c r="A30" s="51"/>
-      <c r="B30" s="51"/>
+      <c r="A30" s="52"/>
+      <c r="B30" s="52"/>
       <c r="C30" s="9">
         <v>16</v>
       </c>
-      <c r="D30" s="51"/>
-      <c r="E30" s="52"/>
-      <c r="F30" s="52"/>
-      <c r="G30" s="52"/>
-      <c r="H30" s="52"/>
+      <c r="D30" s="52"/>
+      <c r="E30" s="53"/>
+      <c r="F30" s="53"/>
+      <c r="G30" s="53"/>
+      <c r="H30" s="53"/>
       <c r="I30" s="17" t="s">
         <v>99</v>
       </c>
@@ -4992,12 +4992,12 @@
       <c r="AA30" s="24"/>
     </row>
     <row r="31" spans="1:27" ht="150" customHeight="1">
-      <c r="A31" s="51"/>
-      <c r="B31" s="51"/>
+      <c r="A31" s="52"/>
+      <c r="B31" s="52"/>
       <c r="C31" s="9">
         <v>17</v>
       </c>
-      <c r="D31" s="51"/>
+      <c r="D31" s="52"/>
       <c r="E31" s="17" t="s">
         <v>100</v>
       </c>
@@ -5037,12 +5037,12 @@
       <c r="AA31" s="24"/>
     </row>
     <row r="32" spans="1:27" ht="150" customHeight="1">
-      <c r="A32" s="51"/>
-      <c r="B32" s="51"/>
+      <c r="A32" s="52"/>
+      <c r="B32" s="52"/>
       <c r="C32" s="9">
         <v>18</v>
       </c>
-      <c r="D32" s="51"/>
+      <c r="D32" s="52"/>
       <c r="E32" s="17" t="s">
         <v>103</v>
       </c>
@@ -5082,12 +5082,12 @@
       <c r="AA32" s="24"/>
     </row>
     <row r="33" spans="1:27" ht="150" customHeight="1">
-      <c r="A33" s="52"/>
-      <c r="B33" s="52"/>
+      <c r="A33" s="53"/>
+      <c r="B33" s="53"/>
       <c r="C33" s="9">
         <v>19</v>
       </c>
-      <c r="D33" s="52"/>
+      <c r="D33" s="53"/>
       <c r="E33" s="17" t="s">
         <v>104</v>
       </c>
@@ -5127,16 +5127,16 @@
       <c r="AA33" s="24"/>
     </row>
     <row r="34" spans="1:27" ht="150" customHeight="1">
-      <c r="A34" s="50" t="s">
+      <c r="A34" s="60" t="s">
         <v>105</v>
       </c>
-      <c r="B34" s="53" t="s">
+      <c r="B34" s="61" t="s">
         <v>106</v>
       </c>
       <c r="C34" s="9">
         <v>1</v>
       </c>
-      <c r="D34" s="50" t="s">
+      <c r="D34" s="60" t="s">
         <v>107</v>
       </c>
       <c r="E34" s="17" t="s">
@@ -5184,12 +5184,12 @@
       <c r="AA34" s="25"/>
     </row>
     <row r="35" spans="1:27" ht="150" customHeight="1">
-      <c r="A35" s="51"/>
-      <c r="B35" s="51"/>
+      <c r="A35" s="52"/>
+      <c r="B35" s="52"/>
       <c r="C35" s="9">
         <v>2</v>
       </c>
-      <c r="D35" s="51"/>
+      <c r="D35" s="52"/>
       <c r="E35" s="17" t="s">
         <v>110</v>
       </c>
@@ -5233,12 +5233,12 @@
       <c r="AA35" s="25"/>
     </row>
     <row r="36" spans="1:27" ht="150" customHeight="1">
-      <c r="A36" s="51"/>
-      <c r="B36" s="51"/>
+      <c r="A36" s="52"/>
+      <c r="B36" s="52"/>
       <c r="C36" s="9">
         <v>3</v>
       </c>
-      <c r="D36" s="51"/>
+      <c r="D36" s="52"/>
       <c r="E36" s="17" t="s">
         <v>112</v>
       </c>
@@ -5280,12 +5280,12 @@
       <c r="AA36" s="25"/>
     </row>
     <row r="37" spans="1:27" ht="150" customHeight="1">
-      <c r="A37" s="51"/>
-      <c r="B37" s="51"/>
+      <c r="A37" s="52"/>
+      <c r="B37" s="52"/>
       <c r="C37" s="9">
         <v>4</v>
       </c>
-      <c r="D37" s="51"/>
+      <c r="D37" s="52"/>
       <c r="E37" s="17" t="s">
         <v>114</v>
       </c>
@@ -5327,12 +5327,12 @@
       <c r="AA37" s="25"/>
     </row>
     <row r="38" spans="1:27" ht="150" customHeight="1">
-      <c r="A38" s="51"/>
-      <c r="B38" s="51"/>
+      <c r="A38" s="52"/>
+      <c r="B38" s="52"/>
       <c r="C38" s="9">
         <v>5</v>
       </c>
-      <c r="D38" s="51"/>
+      <c r="D38" s="52"/>
       <c r="E38" s="17" t="s">
         <v>116</v>
       </c>
@@ -5374,12 +5374,12 @@
       <c r="AA38" s="25"/>
     </row>
     <row r="39" spans="1:27" ht="150" customHeight="1">
-      <c r="A39" s="51"/>
-      <c r="B39" s="51"/>
+      <c r="A39" s="52"/>
+      <c r="B39" s="52"/>
       <c r="C39" s="9">
         <v>6</v>
       </c>
-      <c r="D39" s="51"/>
+      <c r="D39" s="52"/>
       <c r="E39" s="17" t="s">
         <v>118</v>
       </c>
@@ -5421,12 +5421,12 @@
       <c r="AA39" s="25"/>
     </row>
     <row r="40" spans="1:27" ht="150" customHeight="1">
-      <c r="A40" s="51"/>
-      <c r="B40" s="51"/>
+      <c r="A40" s="52"/>
+      <c r="B40" s="52"/>
       <c r="C40" s="9">
         <v>7</v>
       </c>
-      <c r="D40" s="51"/>
+      <c r="D40" s="52"/>
       <c r="E40" s="17" t="s">
         <v>120</v>
       </c>
@@ -5468,12 +5468,12 @@
       <c r="AA40" s="25"/>
     </row>
     <row r="41" spans="1:27" ht="150" customHeight="1">
-      <c r="A41" s="51"/>
-      <c r="B41" s="51"/>
+      <c r="A41" s="52"/>
+      <c r="B41" s="52"/>
       <c r="C41" s="9">
         <v>8</v>
       </c>
-      <c r="D41" s="51"/>
+      <c r="D41" s="52"/>
       <c r="E41" s="17" t="s">
         <v>122</v>
       </c>
@@ -5515,12 +5515,12 @@
       <c r="AA41" s="25"/>
     </row>
     <row r="42" spans="1:27" ht="150" customHeight="1">
-      <c r="A42" s="51"/>
-      <c r="B42" s="51"/>
+      <c r="A42" s="52"/>
+      <c r="B42" s="52"/>
       <c r="C42" s="9">
         <v>9</v>
       </c>
-      <c r="D42" s="51"/>
+      <c r="D42" s="52"/>
       <c r="E42" s="17" t="s">
         <v>123</v>
       </c>
@@ -5562,12 +5562,12 @@
       <c r="AA42" s="25"/>
     </row>
     <row r="43" spans="1:27" ht="150" customHeight="1">
-      <c r="A43" s="51"/>
-      <c r="B43" s="51"/>
+      <c r="A43" s="52"/>
+      <c r="B43" s="52"/>
       <c r="C43" s="9">
         <v>10</v>
       </c>
-      <c r="D43" s="51"/>
+      <c r="D43" s="52"/>
       <c r="E43" s="17" t="s">
         <v>126</v>
       </c>
@@ -5609,12 +5609,12 @@
       <c r="AA43" s="25"/>
     </row>
     <row r="44" spans="1:27" ht="150" customHeight="1">
-      <c r="A44" s="51"/>
-      <c r="B44" s="51"/>
+      <c r="A44" s="52"/>
+      <c r="B44" s="52"/>
       <c r="C44" s="9">
         <v>11</v>
       </c>
-      <c r="D44" s="51"/>
+      <c r="D44" s="52"/>
       <c r="E44" s="17" t="s">
         <v>128</v>
       </c>
@@ -5658,12 +5658,12 @@
       <c r="AA44" s="25"/>
     </row>
     <row r="45" spans="1:27" ht="150" customHeight="1">
-      <c r="A45" s="51"/>
-      <c r="B45" s="51"/>
+      <c r="A45" s="52"/>
+      <c r="B45" s="52"/>
       <c r="C45" s="9">
         <v>12</v>
       </c>
-      <c r="D45" s="51"/>
+      <c r="D45" s="52"/>
       <c r="E45" s="17" t="s">
         <v>130</v>
       </c>
@@ -5707,12 +5707,12 @@
       <c r="AA45" s="25"/>
     </row>
     <row r="46" spans="1:27" ht="150" customHeight="1">
-      <c r="A46" s="51"/>
-      <c r="B46" s="51"/>
+      <c r="A46" s="52"/>
+      <c r="B46" s="52"/>
       <c r="C46" s="9">
         <v>13</v>
       </c>
-      <c r="D46" s="51"/>
+      <c r="D46" s="52"/>
       <c r="E46" s="17" t="s">
         <v>132</v>
       </c>
@@ -5754,12 +5754,12 @@
       <c r="AA46" s="25"/>
     </row>
     <row r="47" spans="1:27" ht="150" customHeight="1">
-      <c r="A47" s="51"/>
-      <c r="B47" s="51"/>
+      <c r="A47" s="52"/>
+      <c r="B47" s="52"/>
       <c r="C47" s="9">
         <v>14</v>
       </c>
-      <c r="D47" s="51"/>
+      <c r="D47" s="52"/>
       <c r="E47" s="17" t="s">
         <v>134</v>
       </c>
@@ -5801,12 +5801,12 @@
       <c r="AA47" s="25"/>
     </row>
     <row r="48" spans="1:27" ht="150" customHeight="1">
-      <c r="A48" s="51"/>
-      <c r="B48" s="51"/>
+      <c r="A48" s="52"/>
+      <c r="B48" s="52"/>
       <c r="C48" s="9">
         <v>15</v>
       </c>
-      <c r="D48" s="51"/>
+      <c r="D48" s="52"/>
       <c r="E48" s="17" t="s">
         <v>136</v>
       </c>
@@ -5848,12 +5848,12 @@
       <c r="AA48" s="25"/>
     </row>
     <row r="49" spans="1:27" ht="150" customHeight="1">
-      <c r="A49" s="51"/>
-      <c r="B49" s="51"/>
+      <c r="A49" s="52"/>
+      <c r="B49" s="52"/>
       <c r="C49" s="9">
         <v>16</v>
       </c>
-      <c r="D49" s="51"/>
+      <c r="D49" s="52"/>
       <c r="E49" s="17" t="s">
         <v>138</v>
       </c>
@@ -5895,16 +5895,16 @@
       <c r="AA49" s="25"/>
     </row>
     <row r="50" spans="1:27" ht="150" customHeight="1">
-      <c r="A50" s="54" t="s">
+      <c r="A50" s="65" t="s">
         <v>140</v>
       </c>
-      <c r="B50" s="57" t="s">
+      <c r="B50" s="66" t="s">
         <v>141</v>
       </c>
       <c r="C50" s="9">
         <v>1</v>
       </c>
-      <c r="D50" s="54" t="s">
+      <c r="D50" s="65" t="s">
         <v>142</v>
       </c>
       <c r="E50" s="17" t="s">
@@ -5948,12 +5948,12 @@
       <c r="AA50" s="25"/>
     </row>
     <row r="51" spans="1:27" ht="150" customHeight="1">
-      <c r="A51" s="51"/>
-      <c r="B51" s="51"/>
+      <c r="A51" s="52"/>
+      <c r="B51" s="52"/>
       <c r="C51" s="9">
         <v>2</v>
       </c>
-      <c r="D51" s="51"/>
+      <c r="D51" s="52"/>
       <c r="E51" s="17" t="s">
         <v>145</v>
       </c>
@@ -5995,12 +5995,12 @@
       <c r="AA51" s="25"/>
     </row>
     <row r="52" spans="1:27" ht="150" customHeight="1">
-      <c r="A52" s="51"/>
-      <c r="B52" s="51"/>
+      <c r="A52" s="52"/>
+      <c r="B52" s="52"/>
       <c r="C52" s="9">
         <v>3</v>
       </c>
-      <c r="D52" s="51"/>
+      <c r="D52" s="52"/>
       <c r="E52" s="17" t="s">
         <v>147</v>
       </c>
@@ -6042,12 +6042,12 @@
       <c r="AA52" s="25"/>
     </row>
     <row r="53" spans="1:27" ht="150" customHeight="1">
-      <c r="A53" s="51"/>
-      <c r="B53" s="51"/>
+      <c r="A53" s="52"/>
+      <c r="B53" s="52"/>
       <c r="C53" s="9">
         <v>4</v>
       </c>
-      <c r="D53" s="51"/>
+      <c r="D53" s="52"/>
       <c r="E53" s="27" t="s">
         <v>149</v>
       </c>
@@ -6089,12 +6089,12 @@
       <c r="AA53" s="25"/>
     </row>
     <row r="54" spans="1:27" ht="150" customHeight="1">
-      <c r="A54" s="51"/>
-      <c r="B54" s="51"/>
+      <c r="A54" s="52"/>
+      <c r="B54" s="52"/>
       <c r="C54" s="9">
         <v>5</v>
       </c>
-      <c r="D54" s="51"/>
+      <c r="D54" s="52"/>
       <c r="E54" s="17" t="s">
         <v>151</v>
       </c>
@@ -6136,12 +6136,12 @@
       <c r="AA54" s="25"/>
     </row>
     <row r="55" spans="1:27" ht="150" customHeight="1">
-      <c r="A55" s="51"/>
-      <c r="B55" s="51"/>
+      <c r="A55" s="52"/>
+      <c r="B55" s="52"/>
       <c r="C55" s="9">
         <v>6</v>
       </c>
-      <c r="D55" s="51"/>
+      <c r="D55" s="52"/>
       <c r="E55" s="17" t="s">
         <v>153</v>
       </c>
@@ -6183,12 +6183,12 @@
       <c r="AA55" s="25"/>
     </row>
     <row r="56" spans="1:27" ht="150" customHeight="1">
-      <c r="A56" s="51"/>
-      <c r="B56" s="51"/>
+      <c r="A56" s="52"/>
+      <c r="B56" s="52"/>
       <c r="C56" s="9">
         <v>7</v>
       </c>
-      <c r="D56" s="51"/>
+      <c r="D56" s="52"/>
       <c r="E56" s="17" t="s">
         <v>155</v>
       </c>
@@ -6230,12 +6230,12 @@
       <c r="AA56" s="25"/>
     </row>
     <row r="57" spans="1:27" ht="150" customHeight="1">
-      <c r="A57" s="51"/>
-      <c r="B57" s="51"/>
+      <c r="A57" s="52"/>
+      <c r="B57" s="52"/>
       <c r="C57" s="9">
         <v>8</v>
       </c>
-      <c r="D57" s="51"/>
+      <c r="D57" s="52"/>
       <c r="E57" s="17" t="s">
         <v>157</v>
       </c>
@@ -6277,12 +6277,12 @@
       <c r="AA57" s="25"/>
     </row>
     <row r="58" spans="1:27" ht="150" customHeight="1">
-      <c r="A58" s="51"/>
-      <c r="B58" s="51"/>
+      <c r="A58" s="52"/>
+      <c r="B58" s="52"/>
       <c r="C58" s="9">
         <v>9</v>
       </c>
-      <c r="D58" s="51"/>
+      <c r="D58" s="52"/>
       <c r="E58" s="17" t="s">
         <v>159</v>
       </c>
@@ -6324,12 +6324,12 @@
       <c r="AA58" s="25"/>
     </row>
     <row r="59" spans="1:27" ht="150" customHeight="1">
-      <c r="A59" s="51"/>
-      <c r="B59" s="51"/>
+      <c r="A59" s="52"/>
+      <c r="B59" s="52"/>
       <c r="C59" s="9">
         <v>10</v>
       </c>
-      <c r="D59" s="51"/>
+      <c r="D59" s="52"/>
       <c r="E59" s="17" t="s">
         <v>161</v>
       </c>
@@ -6371,12 +6371,12 @@
       <c r="AA59" s="25"/>
     </row>
     <row r="60" spans="1:27" ht="150" customHeight="1">
-      <c r="A60" s="51"/>
-      <c r="B60" s="51"/>
+      <c r="A60" s="52"/>
+      <c r="B60" s="52"/>
       <c r="C60" s="9">
         <v>11</v>
       </c>
-      <c r="D60" s="51"/>
+      <c r="D60" s="52"/>
       <c r="E60" s="17" t="s">
         <v>163</v>
       </c>
@@ -6418,12 +6418,12 @@
       <c r="AA60" s="25"/>
     </row>
     <row r="61" spans="1:27" ht="150" customHeight="1">
-      <c r="A61" s="51"/>
-      <c r="B61" s="51"/>
+      <c r="A61" s="52"/>
+      <c r="B61" s="52"/>
       <c r="C61" s="9">
         <v>12</v>
       </c>
-      <c r="D61" s="51"/>
+      <c r="D61" s="52"/>
       <c r="E61" s="17" t="s">
         <v>165</v>
       </c>
@@ -6465,12 +6465,12 @@
       <c r="AA61" s="25"/>
     </row>
     <row r="62" spans="1:27" ht="150" customHeight="1">
-      <c r="A62" s="51"/>
-      <c r="B62" s="51"/>
+      <c r="A62" s="52"/>
+      <c r="B62" s="52"/>
       <c r="C62" s="9">
         <v>13</v>
       </c>
-      <c r="D62" s="51"/>
+      <c r="D62" s="52"/>
       <c r="E62" s="17" t="s">
         <v>167</v>
       </c>
@@ -6512,12 +6512,12 @@
       <c r="AA62" s="25"/>
     </row>
     <row r="63" spans="1:27" ht="150" customHeight="1">
-      <c r="A63" s="51"/>
-      <c r="B63" s="51"/>
+      <c r="A63" s="52"/>
+      <c r="B63" s="52"/>
       <c r="C63" s="9">
         <v>14</v>
       </c>
-      <c r="D63" s="51"/>
+      <c r="D63" s="52"/>
       <c r="E63" s="17" t="s">
         <v>169</v>
       </c>
@@ -6559,12 +6559,12 @@
       <c r="AA63" s="25"/>
     </row>
     <row r="64" spans="1:27" ht="150" customHeight="1">
-      <c r="A64" s="51"/>
-      <c r="B64" s="51"/>
+      <c r="A64" s="52"/>
+      <c r="B64" s="52"/>
       <c r="C64" s="9">
         <v>15</v>
       </c>
-      <c r="D64" s="51"/>
+      <c r="D64" s="52"/>
       <c r="E64" s="17" t="s">
         <v>171</v>
       </c>
@@ -6606,12 +6606,12 @@
       <c r="AA64" s="25"/>
     </row>
     <row r="65" spans="1:27" ht="150" customHeight="1">
-      <c r="A65" s="52"/>
-      <c r="B65" s="52"/>
+      <c r="A65" s="53"/>
+      <c r="B65" s="53"/>
       <c r="C65" s="9">
         <v>16</v>
       </c>
-      <c r="D65" s="52"/>
+      <c r="D65" s="53"/>
       <c r="E65" s="17" t="s">
         <v>173</v>
       </c>
@@ -6653,16 +6653,16 @@
       <c r="AA65" s="25"/>
     </row>
     <row r="66" spans="1:27" ht="150" customHeight="1">
-      <c r="A66" s="50" t="s">
+      <c r="A66" s="60" t="s">
         <v>175</v>
       </c>
-      <c r="B66" s="53" t="s">
+      <c r="B66" s="61" t="s">
         <v>176</v>
       </c>
       <c r="C66" s="9">
         <v>1</v>
       </c>
-      <c r="D66" s="50" t="s">
+      <c r="D66" s="60" t="s">
         <v>177</v>
       </c>
       <c r="E66" s="17" t="s">
@@ -6706,12 +6706,12 @@
       <c r="AA66" s="25"/>
     </row>
     <row r="67" spans="1:27" ht="150" customHeight="1">
-      <c r="A67" s="51"/>
-      <c r="B67" s="51"/>
+      <c r="A67" s="52"/>
+      <c r="B67" s="52"/>
       <c r="C67" s="9">
         <v>2</v>
       </c>
-      <c r="D67" s="51"/>
+      <c r="D67" s="52"/>
       <c r="E67" s="17" t="s">
         <v>180</v>
       </c>
@@ -6753,12 +6753,12 @@
       <c r="AA67" s="25"/>
     </row>
     <row r="68" spans="1:27" ht="150" customHeight="1">
-      <c r="A68" s="51"/>
-      <c r="B68" s="51"/>
+      <c r="A68" s="52"/>
+      <c r="B68" s="52"/>
       <c r="C68" s="9">
         <v>3</v>
       </c>
-      <c r="D68" s="51"/>
+      <c r="D68" s="52"/>
       <c r="E68" s="17" t="s">
         <v>182</v>
       </c>
@@ -6800,12 +6800,12 @@
       <c r="AA68" s="25"/>
     </row>
     <row r="69" spans="1:27" ht="150" customHeight="1">
-      <c r="A69" s="51"/>
-      <c r="B69" s="51"/>
+      <c r="A69" s="52"/>
+      <c r="B69" s="52"/>
       <c r="C69" s="9">
         <v>4</v>
       </c>
-      <c r="D69" s="51"/>
+      <c r="D69" s="52"/>
       <c r="E69" s="17" t="s">
         <v>184</v>
       </c>
@@ -6847,12 +6847,12 @@
       <c r="AA69" s="25"/>
     </row>
     <row r="70" spans="1:27" ht="150" customHeight="1">
-      <c r="A70" s="51"/>
-      <c r="B70" s="51"/>
+      <c r="A70" s="52"/>
+      <c r="B70" s="52"/>
       <c r="C70" s="9">
         <v>5</v>
       </c>
-      <c r="D70" s="51"/>
+      <c r="D70" s="52"/>
       <c r="E70" s="17" t="s">
         <v>186</v>
       </c>
@@ -6894,12 +6894,12 @@
       <c r="AA70" s="25"/>
     </row>
     <row r="71" spans="1:27" ht="150" customHeight="1">
-      <c r="A71" s="52"/>
-      <c r="B71" s="52"/>
+      <c r="A71" s="53"/>
+      <c r="B71" s="53"/>
       <c r="C71" s="9">
         <v>6</v>
       </c>
-      <c r="D71" s="52"/>
+      <c r="D71" s="53"/>
       <c r="E71" s="17" t="s">
         <v>188</v>
       </c>
@@ -6941,28 +6941,28 @@
       <c r="AA71" s="25"/>
     </row>
     <row r="72" spans="1:27" ht="150" customHeight="1">
-      <c r="A72" s="50" t="s">
+      <c r="A72" s="60" t="s">
         <v>190</v>
       </c>
-      <c r="B72" s="53" t="s">
+      <c r="B72" s="61" t="s">
         <v>191</v>
       </c>
       <c r="C72" s="9">
         <v>1</v>
       </c>
-      <c r="D72" s="50" t="s">
+      <c r="D72" s="60" t="s">
         <v>192</v>
       </c>
-      <c r="E72" s="50" t="s">
+      <c r="E72" s="60" t="s">
         <v>193</v>
       </c>
-      <c r="F72" s="53" t="s">
+      <c r="F72" s="61" t="s">
         <v>22</v>
       </c>
       <c r="G72" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="H72" s="50" t="s">
+      <c r="H72" s="60" t="s">
         <v>194</v>
       </c>
       <c r="I72" s="17" t="s">
@@ -6994,16 +6994,16 @@
       <c r="AA72" s="24"/>
     </row>
     <row r="73" spans="1:27" ht="150" customHeight="1">
-      <c r="A73" s="51"/>
-      <c r="B73" s="51"/>
+      <c r="A73" s="52"/>
+      <c r="B73" s="52"/>
       <c r="C73" s="9">
         <v>2</v>
       </c>
-      <c r="D73" s="51"/>
-      <c r="E73" s="51"/>
-      <c r="F73" s="52"/>
+      <c r="D73" s="52"/>
+      <c r="E73" s="52"/>
+      <c r="F73" s="53"/>
       <c r="G73" s="18"/>
-      <c r="H73" s="52"/>
+      <c r="H73" s="53"/>
       <c r="I73" s="17" t="s">
         <v>196</v>
       </c>
@@ -7033,13 +7033,13 @@
       <c r="AA73" s="24"/>
     </row>
     <row r="74" spans="1:27" ht="150" customHeight="1">
-      <c r="A74" s="51"/>
-      <c r="B74" s="51"/>
+      <c r="A74" s="52"/>
+      <c r="B74" s="52"/>
       <c r="C74" s="9">
         <v>3</v>
       </c>
-      <c r="D74" s="51"/>
-      <c r="E74" s="51"/>
+      <c r="D74" s="52"/>
+      <c r="E74" s="52"/>
       <c r="F74" s="18" t="s">
         <v>22</v>
       </c>
@@ -7078,13 +7078,13 @@
       <c r="AA74" s="24"/>
     </row>
     <row r="75" spans="1:27" ht="150" customHeight="1">
-      <c r="A75" s="51"/>
-      <c r="B75" s="51"/>
+      <c r="A75" s="52"/>
+      <c r="B75" s="52"/>
       <c r="C75" s="9">
         <v>4</v>
       </c>
-      <c r="D75" s="51"/>
-      <c r="E75" s="52"/>
+      <c r="D75" s="52"/>
+      <c r="E75" s="53"/>
       <c r="F75" s="18" t="s">
         <v>22</v>
       </c>
@@ -7123,12 +7123,12 @@
       <c r="AA75" s="24"/>
     </row>
     <row r="76" spans="1:27" ht="150" customHeight="1">
-      <c r="A76" s="51"/>
-      <c r="B76" s="51"/>
+      <c r="A76" s="52"/>
+      <c r="B76" s="52"/>
       <c r="C76" s="9">
         <v>5</v>
       </c>
-      <c r="D76" s="51"/>
+      <c r="D76" s="52"/>
       <c r="E76" s="26" t="s">
         <v>201</v>
       </c>
@@ -7170,12 +7170,12 @@
       <c r="AA76" s="24"/>
     </row>
     <row r="77" spans="1:27" ht="150" customHeight="1">
-      <c r="A77" s="51"/>
-      <c r="B77" s="51"/>
+      <c r="A77" s="52"/>
+      <c r="B77" s="52"/>
       <c r="C77" s="9">
         <v>6</v>
       </c>
-      <c r="D77" s="51"/>
+      <c r="D77" s="52"/>
       <c r="E77" s="26" t="s">
         <v>204</v>
       </c>
@@ -7217,12 +7217,12 @@
       <c r="AA77" s="24"/>
     </row>
     <row r="78" spans="1:27" ht="150" customHeight="1">
-      <c r="A78" s="51"/>
-      <c r="B78" s="51"/>
+      <c r="A78" s="52"/>
+      <c r="B78" s="52"/>
       <c r="C78" s="9">
         <v>7</v>
       </c>
-      <c r="D78" s="51"/>
+      <c r="D78" s="52"/>
       <c r="E78" s="26" t="s">
         <v>206</v>
       </c>
@@ -7264,12 +7264,12 @@
       <c r="AA78" s="24"/>
     </row>
     <row r="79" spans="1:27" ht="150" customHeight="1">
-      <c r="A79" s="51"/>
-      <c r="B79" s="51"/>
+      <c r="A79" s="52"/>
+      <c r="B79" s="52"/>
       <c r="C79" s="9">
         <v>8</v>
       </c>
-      <c r="D79" s="51"/>
+      <c r="D79" s="52"/>
       <c r="E79" s="26" t="s">
         <v>208</v>
       </c>
@@ -7311,12 +7311,12 @@
       <c r="AA79" s="24"/>
     </row>
     <row r="80" spans="1:27" ht="150" customHeight="1">
-      <c r="A80" s="52"/>
-      <c r="B80" s="52"/>
+      <c r="A80" s="53"/>
+      <c r="B80" s="53"/>
       <c r="C80" s="9">
         <v>9</v>
       </c>
-      <c r="D80" s="52"/>
+      <c r="D80" s="53"/>
       <c r="E80" s="26" t="s">
         <v>210</v>
       </c>
@@ -7358,16 +7358,16 @@
       <c r="AA80" s="24"/>
     </row>
     <row r="81" spans="1:27" ht="150" customHeight="1">
-      <c r="A81" s="50" t="s">
+      <c r="A81" s="60" t="s">
         <v>212</v>
       </c>
-      <c r="B81" s="53" t="s">
+      <c r="B81" s="61" t="s">
         <v>213</v>
       </c>
       <c r="C81" s="19">
         <v>1</v>
       </c>
-      <c r="D81" s="50" t="s">
+      <c r="D81" s="60" t="s">
         <v>214</v>
       </c>
       <c r="E81" s="26" t="s">
@@ -7388,7 +7388,7 @@
       <c r="J81" s="19"/>
       <c r="K81" s="19"/>
       <c r="L81" s="20"/>
-      <c r="M81" s="56" t="s">
+      <c r="M81" s="63" t="s">
         <v>218</v>
       </c>
       <c r="N81" s="21"/>
@@ -7411,12 +7411,12 @@
       <c r="AA81" s="24"/>
     </row>
     <row r="82" spans="1:27" ht="150" customHeight="1">
-      <c r="A82" s="52"/>
-      <c r="B82" s="52"/>
+      <c r="A82" s="53"/>
+      <c r="B82" s="53"/>
       <c r="C82" s="19">
         <v>2</v>
       </c>
-      <c r="D82" s="52"/>
+      <c r="D82" s="53"/>
       <c r="E82" s="26" t="s">
         <v>219</v>
       </c>
@@ -7435,7 +7435,7 @@
       <c r="J82" s="19"/>
       <c r="K82" s="19"/>
       <c r="L82" s="20"/>
-      <c r="M82" s="52"/>
+      <c r="M82" s="53"/>
       <c r="N82" s="24"/>
       <c r="O82" s="22"/>
       <c r="P82" s="19"/>
@@ -7477,16 +7477,16 @@
       <c r="R83" s="14"/>
     </row>
     <row r="84" spans="1:27" ht="150" customHeight="1">
-      <c r="A84" s="50" t="s">
+      <c r="A84" s="60" t="s">
         <v>223</v>
       </c>
-      <c r="B84" s="53" t="s">
+      <c r="B84" s="61" t="s">
         <v>224</v>
       </c>
       <c r="C84" s="19">
         <v>1</v>
       </c>
-      <c r="D84" s="50" t="s">
+      <c r="D84" s="60" t="s">
         <v>223</v>
       </c>
       <c r="E84" s="26" t="s">
@@ -7528,12 +7528,12 @@
       <c r="AA84" s="24"/>
     </row>
     <row r="85" spans="1:27" ht="150" customHeight="1">
-      <c r="A85" s="51"/>
-      <c r="B85" s="51"/>
+      <c r="A85" s="52"/>
+      <c r="B85" s="52"/>
       <c r="C85" s="19">
         <v>2</v>
       </c>
-      <c r="D85" s="51"/>
+      <c r="D85" s="52"/>
       <c r="E85" s="26" t="s">
         <v>228</v>
       </c>
@@ -7575,12 +7575,12 @@
       <c r="AA85" s="24"/>
     </row>
     <row r="86" spans="1:27" ht="150" customHeight="1">
-      <c r="A86" s="51"/>
-      <c r="B86" s="51"/>
+      <c r="A86" s="52"/>
+      <c r="B86" s="52"/>
       <c r="C86" s="19">
         <v>3</v>
       </c>
-      <c r="D86" s="51"/>
+      <c r="D86" s="52"/>
       <c r="E86" s="26" t="s">
         <v>231</v>
       </c>
@@ -7622,12 +7622,12 @@
       <c r="AA86" s="24"/>
     </row>
     <row r="87" spans="1:27" ht="150" customHeight="1">
-      <c r="A87" s="51"/>
-      <c r="B87" s="51"/>
+      <c r="A87" s="52"/>
+      <c r="B87" s="52"/>
       <c r="C87" s="19">
         <v>4</v>
       </c>
-      <c r="D87" s="51"/>
+      <c r="D87" s="52"/>
       <c r="E87" s="26" t="s">
         <v>234</v>
       </c>
@@ -7669,12 +7669,12 @@
       <c r="AA87" s="24"/>
     </row>
     <row r="88" spans="1:27" ht="150" customHeight="1">
-      <c r="A88" s="51"/>
-      <c r="B88" s="51"/>
+      <c r="A88" s="52"/>
+      <c r="B88" s="52"/>
       <c r="C88" s="19">
         <v>5</v>
       </c>
-      <c r="D88" s="51"/>
+      <c r="D88" s="52"/>
       <c r="E88" s="26" t="s">
         <v>237</v>
       </c>
@@ -7718,19 +7718,19 @@
       <c r="AA88" s="24"/>
     </row>
     <row r="89" spans="1:27" ht="150" customHeight="1">
-      <c r="A89" s="51"/>
-      <c r="B89" s="51"/>
+      <c r="A89" s="52"/>
+      <c r="B89" s="52"/>
       <c r="C89" s="19">
         <v>6</v>
       </c>
-      <c r="D89" s="51"/>
-      <c r="E89" s="50" t="s">
+      <c r="D89" s="52"/>
+      <c r="E89" s="60" t="s">
         <v>240</v>
       </c>
-      <c r="F89" s="53" t="s">
+      <c r="F89" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="G89" s="58" t="s">
+      <c r="G89" s="64" t="s">
         <v>66</v>
       </c>
       <c r="H89" s="17" t="s">
@@ -7765,15 +7765,15 @@
       <c r="AA89" s="24"/>
     </row>
     <row r="90" spans="1:27" ht="150" customHeight="1">
-      <c r="A90" s="51"/>
-      <c r="B90" s="51"/>
+      <c r="A90" s="52"/>
+      <c r="B90" s="52"/>
       <c r="C90" s="19">
         <v>7</v>
       </c>
-      <c r="D90" s="51"/>
-      <c r="E90" s="52"/>
-      <c r="F90" s="52"/>
-      <c r="G90" s="52"/>
+      <c r="D90" s="52"/>
+      <c r="E90" s="53"/>
+      <c r="F90" s="53"/>
+      <c r="G90" s="53"/>
       <c r="H90" s="17" t="s">
         <v>243</v>
       </c>
@@ -7806,12 +7806,12 @@
       <c r="AA90" s="24"/>
     </row>
     <row r="91" spans="1:27" ht="150" customHeight="1">
-      <c r="A91" s="51"/>
-      <c r="B91" s="51"/>
+      <c r="A91" s="52"/>
+      <c r="B91" s="52"/>
       <c r="C91" s="19">
         <v>8</v>
       </c>
-      <c r="D91" s="51"/>
+      <c r="D91" s="52"/>
       <c r="E91" s="26" t="s">
         <v>245</v>
       </c>
@@ -7851,12 +7851,12 @@
       <c r="AA91" s="24"/>
     </row>
     <row r="92" spans="1:27" ht="150" customHeight="1">
-      <c r="A92" s="51"/>
-      <c r="B92" s="51"/>
+      <c r="A92" s="52"/>
+      <c r="B92" s="52"/>
       <c r="C92" s="19">
         <v>9</v>
       </c>
-      <c r="D92" s="51"/>
+      <c r="D92" s="52"/>
       <c r="E92" s="26" t="s">
         <v>248</v>
       </c>
@@ -7896,12 +7896,12 @@
       <c r="AA92" s="24"/>
     </row>
     <row r="93" spans="1:27" ht="150" customHeight="1">
-      <c r="A93" s="52"/>
-      <c r="B93" s="52"/>
+      <c r="A93" s="53"/>
+      <c r="B93" s="53"/>
       <c r="C93" s="19">
         <v>10</v>
       </c>
-      <c r="D93" s="52"/>
+      <c r="D93" s="53"/>
       <c r="E93" s="26" t="s">
         <v>251</v>
       </c>
@@ -7934,16 +7934,16 @@
       </c>
     </row>
     <row r="94" spans="1:27" ht="150" customHeight="1">
-      <c r="A94" s="50" t="s">
+      <c r="A94" s="60" t="s">
         <v>254</v>
       </c>
-      <c r="B94" s="53" t="s">
+      <c r="B94" s="61" t="s">
         <v>255</v>
       </c>
       <c r="C94" s="19">
         <v>1</v>
       </c>
-      <c r="D94" s="50" t="s">
+      <c r="D94" s="60" t="s">
         <v>256</v>
       </c>
       <c r="E94" s="26" t="s">
@@ -7980,12 +7980,12 @@
       </c>
     </row>
     <row r="95" spans="1:27" ht="150" customHeight="1">
-      <c r="A95" s="52"/>
-      <c r="B95" s="52"/>
+      <c r="A95" s="53"/>
+      <c r="B95" s="53"/>
       <c r="C95" s="19">
         <v>2</v>
       </c>
-      <c r="D95" s="52"/>
+      <c r="D95" s="53"/>
       <c r="E95" s="26" t="s">
         <v>260</v>
       </c>
@@ -8020,19 +8020,19 @@
       </c>
     </row>
     <row r="96" spans="1:27" ht="150" customHeight="1">
-      <c r="A96" s="59" t="s">
+      <c r="A96" s="62" t="s">
         <v>262</v>
       </c>
-      <c r="B96" s="60" t="s">
+      <c r="B96" s="54" t="s">
         <v>263</v>
       </c>
       <c r="C96" s="9">
         <v>1</v>
       </c>
-      <c r="D96" s="55" t="s">
+      <c r="D96" s="51" t="s">
         <v>264</v>
       </c>
-      <c r="E96" s="55" t="s">
+      <c r="E96" s="51" t="s">
         <v>265</v>
       </c>
       <c r="F96" s="14" t="s">
@@ -8064,13 +8064,13 @@
       </c>
     </row>
     <row r="97" spans="1:18" ht="150" customHeight="1">
-      <c r="A97" s="51"/>
-      <c r="B97" s="51"/>
+      <c r="A97" s="52"/>
+      <c r="B97" s="52"/>
       <c r="C97" s="9">
         <v>2</v>
       </c>
-      <c r="D97" s="51"/>
-      <c r="E97" s="52"/>
+      <c r="D97" s="52"/>
+      <c r="E97" s="53"/>
       <c r="F97" s="14" t="s">
         <v>266</v>
       </c>
@@ -8100,13 +8100,13 @@
       </c>
     </row>
     <row r="98" spans="1:18" ht="150" customHeight="1">
-      <c r="A98" s="51"/>
-      <c r="B98" s="51"/>
+      <c r="A98" s="52"/>
+      <c r="B98" s="52"/>
       <c r="C98" s="9">
         <v>3</v>
       </c>
-      <c r="D98" s="51"/>
-      <c r="E98" s="55" t="s">
+      <c r="D98" s="52"/>
+      <c r="E98" s="51" t="s">
         <v>271</v>
       </c>
       <c r="F98" s="14" t="s">
@@ -8138,13 +8138,13 @@
       </c>
     </row>
     <row r="99" spans="1:18" ht="150" customHeight="1">
-      <c r="A99" s="51"/>
-      <c r="B99" s="51"/>
+      <c r="A99" s="52"/>
+      <c r="B99" s="52"/>
       <c r="C99" s="9">
         <v>4</v>
       </c>
-      <c r="D99" s="51"/>
-      <c r="E99" s="52"/>
+      <c r="D99" s="52"/>
+      <c r="E99" s="53"/>
       <c r="F99" s="14" t="s">
         <v>266</v>
       </c>
@@ -8174,13 +8174,13 @@
       </c>
     </row>
     <row r="100" spans="1:18" ht="150" customHeight="1">
-      <c r="A100" s="51"/>
-      <c r="B100" s="51"/>
+      <c r="A100" s="52"/>
+      <c r="B100" s="52"/>
       <c r="C100" s="9">
         <v>5</v>
       </c>
-      <c r="D100" s="51"/>
-      <c r="E100" s="55" t="s">
+      <c r="D100" s="52"/>
+      <c r="E100" s="51" t="s">
         <v>273</v>
       </c>
       <c r="F100" s="14" t="s">
@@ -8212,13 +8212,13 @@
       </c>
     </row>
     <row r="101" spans="1:18" ht="150" customHeight="1">
-      <c r="A101" s="51"/>
-      <c r="B101" s="51"/>
+      <c r="A101" s="52"/>
+      <c r="B101" s="52"/>
       <c r="C101" s="9">
         <v>6</v>
       </c>
-      <c r="D101" s="51"/>
-      <c r="E101" s="52"/>
+      <c r="D101" s="52"/>
+      <c r="E101" s="53"/>
       <c r="F101" s="14" t="s">
         <v>266</v>
       </c>
@@ -8248,13 +8248,13 @@
       </c>
     </row>
     <row r="102" spans="1:18" ht="150" customHeight="1">
-      <c r="A102" s="51"/>
-      <c r="B102" s="51"/>
+      <c r="A102" s="52"/>
+      <c r="B102" s="52"/>
       <c r="C102" s="9">
         <v>7</v>
       </c>
-      <c r="D102" s="51"/>
-      <c r="E102" s="55" t="s">
+      <c r="D102" s="52"/>
+      <c r="E102" s="51" t="s">
         <v>275</v>
       </c>
       <c r="F102" s="14" t="s">
@@ -8286,13 +8286,13 @@
       </c>
     </row>
     <row r="103" spans="1:18" ht="150" customHeight="1">
-      <c r="A103" s="51"/>
-      <c r="B103" s="52"/>
+      <c r="A103" s="52"/>
+      <c r="B103" s="53"/>
       <c r="C103" s="9">
         <v>8</v>
       </c>
-      <c r="D103" s="52"/>
-      <c r="E103" s="51"/>
+      <c r="D103" s="53"/>
+      <c r="E103" s="52"/>
       <c r="F103" s="14" t="s">
         <v>266</v>
       </c>
@@ -8322,17 +8322,17 @@
       </c>
     </row>
     <row r="104" spans="1:18" ht="150" customHeight="1">
-      <c r="A104" s="51"/>
-      <c r="B104" s="60" t="s">
+      <c r="A104" s="52"/>
+      <c r="B104" s="54" t="s">
         <v>278</v>
       </c>
       <c r="C104" s="9">
         <v>1</v>
       </c>
-      <c r="D104" s="55" t="s">
+      <c r="D104" s="51" t="s">
         <v>279</v>
       </c>
-      <c r="E104" s="55" t="s">
+      <c r="E104" s="51" t="s">
         <v>265</v>
       </c>
       <c r="F104" s="14" t="s">
@@ -8364,13 +8364,13 @@
       </c>
     </row>
     <row r="105" spans="1:18" ht="150" customHeight="1">
-      <c r="A105" s="51"/>
-      <c r="B105" s="51"/>
+      <c r="A105" s="52"/>
+      <c r="B105" s="52"/>
       <c r="C105" s="9">
         <v>2</v>
       </c>
-      <c r="D105" s="51"/>
-      <c r="E105" s="52"/>
+      <c r="D105" s="52"/>
+      <c r="E105" s="53"/>
       <c r="F105" s="14" t="s">
         <v>266</v>
       </c>
@@ -8400,13 +8400,13 @@
       </c>
     </row>
     <row r="106" spans="1:18" ht="150" customHeight="1">
-      <c r="A106" s="51"/>
-      <c r="B106" s="51"/>
+      <c r="A106" s="52"/>
+      <c r="B106" s="52"/>
       <c r="C106" s="9">
         <v>3</v>
       </c>
-      <c r="D106" s="51"/>
-      <c r="E106" s="55" t="s">
+      <c r="D106" s="52"/>
+      <c r="E106" s="51" t="s">
         <v>271</v>
       </c>
       <c r="F106" s="14" t="s">
@@ -8438,13 +8438,13 @@
       </c>
     </row>
     <row r="107" spans="1:18" ht="150" customHeight="1">
-      <c r="A107" s="51"/>
-      <c r="B107" s="51"/>
+      <c r="A107" s="52"/>
+      <c r="B107" s="52"/>
       <c r="C107" s="9">
         <v>4</v>
       </c>
-      <c r="D107" s="51"/>
-      <c r="E107" s="52"/>
+      <c r="D107" s="52"/>
+      <c r="E107" s="53"/>
       <c r="F107" s="14" t="s">
         <v>266</v>
       </c>
@@ -8474,13 +8474,13 @@
       </c>
     </row>
     <row r="108" spans="1:18" ht="150" customHeight="1">
-      <c r="A108" s="51"/>
-      <c r="B108" s="51"/>
+      <c r="A108" s="52"/>
+      <c r="B108" s="52"/>
       <c r="C108" s="9">
         <v>5</v>
       </c>
-      <c r="D108" s="51"/>
-      <c r="E108" s="55" t="s">
+      <c r="D108" s="52"/>
+      <c r="E108" s="51" t="s">
         <v>273</v>
       </c>
       <c r="F108" s="14" t="s">
@@ -8512,13 +8512,13 @@
       </c>
     </row>
     <row r="109" spans="1:18" ht="150" customHeight="1">
-      <c r="A109" s="51"/>
-      <c r="B109" s="51"/>
+      <c r="A109" s="52"/>
+      <c r="B109" s="52"/>
       <c r="C109" s="9">
         <v>6</v>
       </c>
-      <c r="D109" s="51"/>
-      <c r="E109" s="52"/>
+      <c r="D109" s="52"/>
+      <c r="E109" s="53"/>
       <c r="F109" s="14" t="s">
         <v>266</v>
       </c>
@@ -8548,13 +8548,13 @@
       </c>
     </row>
     <row r="110" spans="1:18" ht="150" customHeight="1">
-      <c r="A110" s="51"/>
-      <c r="B110" s="51"/>
+      <c r="A110" s="52"/>
+      <c r="B110" s="52"/>
       <c r="C110" s="9">
         <v>7</v>
       </c>
-      <c r="D110" s="51"/>
-      <c r="E110" s="55" t="s">
+      <c r="D110" s="52"/>
+      <c r="E110" s="51" t="s">
         <v>275</v>
       </c>
       <c r="F110" s="14" t="s">
@@ -8586,13 +8586,13 @@
       </c>
     </row>
     <row r="111" spans="1:18" ht="150" customHeight="1">
-      <c r="A111" s="51"/>
-      <c r="B111" s="52"/>
+      <c r="A111" s="52"/>
+      <c r="B111" s="53"/>
       <c r="C111" s="9">
         <v>8</v>
       </c>
-      <c r="D111" s="52"/>
-      <c r="E111" s="51"/>
+      <c r="D111" s="53"/>
+      <c r="E111" s="52"/>
       <c r="F111" s="14" t="s">
         <v>266</v>
       </c>
@@ -8622,14 +8622,14 @@
       </c>
     </row>
     <row r="112" spans="1:18" ht="150" customHeight="1">
-      <c r="A112" s="51"/>
-      <c r="B112" s="60" t="s">
+      <c r="A112" s="52"/>
+      <c r="B112" s="54" t="s">
         <v>282</v>
       </c>
       <c r="C112" s="9">
         <v>1</v>
       </c>
-      <c r="D112" s="55" t="s">
+      <c r="D112" s="51" t="s">
         <v>283</v>
       </c>
       <c r="E112" s="29" t="s">
@@ -8664,12 +8664,12 @@
       </c>
     </row>
     <row r="113" spans="1:18" ht="150" customHeight="1">
-      <c r="A113" s="51"/>
-      <c r="B113" s="51"/>
+      <c r="A113" s="52"/>
+      <c r="B113" s="52"/>
       <c r="C113" s="9">
         <v>2</v>
       </c>
-      <c r="D113" s="51"/>
+      <c r="D113" s="52"/>
       <c r="E113" s="29" t="s">
         <v>287</v>
       </c>
@@ -8702,12 +8702,12 @@
       </c>
     </row>
     <row r="114" spans="1:18" ht="150" customHeight="1">
-      <c r="A114" s="51"/>
-      <c r="B114" s="51"/>
+      <c r="A114" s="52"/>
+      <c r="B114" s="52"/>
       <c r="C114" s="9">
         <v>3</v>
       </c>
-      <c r="D114" s="51"/>
+      <c r="D114" s="52"/>
       <c r="E114" s="29" t="s">
         <v>290</v>
       </c>
@@ -8740,12 +8740,12 @@
       </c>
     </row>
     <row r="115" spans="1:18" ht="150" customHeight="1">
-      <c r="A115" s="51"/>
-      <c r="B115" s="51"/>
+      <c r="A115" s="52"/>
+      <c r="B115" s="52"/>
       <c r="C115" s="9">
         <v>4</v>
       </c>
-      <c r="D115" s="51"/>
+      <c r="D115" s="52"/>
       <c r="E115" s="29" t="s">
         <v>292</v>
       </c>
@@ -8778,12 +8778,12 @@
       </c>
     </row>
     <row r="116" spans="1:18" ht="150" customHeight="1">
-      <c r="A116" s="51"/>
-      <c r="B116" s="51"/>
+      <c r="A116" s="52"/>
+      <c r="B116" s="52"/>
       <c r="C116" s="9">
         <v>5</v>
       </c>
-      <c r="D116" s="51"/>
+      <c r="D116" s="52"/>
       <c r="E116" s="29" t="s">
         <v>294</v>
       </c>
@@ -8816,12 +8816,12 @@
       </c>
     </row>
     <row r="117" spans="1:18" ht="150" customHeight="1">
-      <c r="A117" s="51"/>
-      <c r="B117" s="51"/>
+      <c r="A117" s="52"/>
+      <c r="B117" s="52"/>
       <c r="C117" s="9">
         <v>6</v>
       </c>
-      <c r="D117" s="51"/>
+      <c r="D117" s="52"/>
       <c r="E117" s="29" t="s">
         <v>296</v>
       </c>
@@ -8854,12 +8854,12 @@
       </c>
     </row>
     <row r="118" spans="1:18" ht="150" customHeight="1">
-      <c r="A118" s="51"/>
-      <c r="B118" s="51"/>
+      <c r="A118" s="52"/>
+      <c r="B118" s="52"/>
       <c r="C118" s="9">
         <v>7</v>
       </c>
-      <c r="D118" s="51"/>
+      <c r="D118" s="52"/>
       <c r="E118" s="29" t="s">
         <v>298</v>
       </c>
@@ -8892,12 +8892,12 @@
       </c>
     </row>
     <row r="119" spans="1:18" ht="150" customHeight="1">
-      <c r="A119" s="51"/>
-      <c r="B119" s="51"/>
+      <c r="A119" s="52"/>
+      <c r="B119" s="52"/>
       <c r="C119" s="9">
         <v>8</v>
       </c>
-      <c r="D119" s="51"/>
+      <c r="D119" s="52"/>
       <c r="E119" s="29" t="s">
         <v>300</v>
       </c>
@@ -8930,13 +8930,13 @@
       </c>
     </row>
     <row r="120" spans="1:18" ht="150" customHeight="1">
-      <c r="A120" s="51"/>
-      <c r="B120" s="51"/>
+      <c r="A120" s="52"/>
+      <c r="B120" s="52"/>
       <c r="C120" s="9">
         <v>9</v>
       </c>
-      <c r="D120" s="51"/>
-      <c r="E120" s="55" t="s">
+      <c r="D120" s="52"/>
+      <c r="E120" s="51" t="s">
         <v>302</v>
       </c>
       <c r="F120" s="14" t="s">
@@ -8945,7 +8945,7 @@
       <c r="G120" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="H120" s="55" t="s">
+      <c r="H120" s="51" t="s">
         <v>303</v>
       </c>
       <c r="I120" s="10" t="s">
@@ -8968,20 +8968,20 @@
       </c>
     </row>
     <row r="121" spans="1:18" ht="150" customHeight="1">
-      <c r="A121" s="51"/>
-      <c r="B121" s="51"/>
+      <c r="A121" s="52"/>
+      <c r="B121" s="52"/>
       <c r="C121" s="9">
         <v>10</v>
       </c>
-      <c r="D121" s="51"/>
-      <c r="E121" s="51"/>
+      <c r="D121" s="52"/>
+      <c r="E121" s="52"/>
       <c r="F121" s="14" t="s">
         <v>266</v>
       </c>
       <c r="G121" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="H121" s="52"/>
+      <c r="H121" s="53"/>
       <c r="I121" s="10" t="s">
         <v>304</v>
       </c>
@@ -9002,13 +9002,13 @@
       </c>
     </row>
     <row r="122" spans="1:18" ht="150" customHeight="1">
-      <c r="A122" s="51"/>
-      <c r="B122" s="51"/>
+      <c r="A122" s="52"/>
+      <c r="B122" s="52"/>
       <c r="C122" s="9">
         <v>11</v>
       </c>
-      <c r="D122" s="51"/>
-      <c r="E122" s="51"/>
+      <c r="D122" s="52"/>
+      <c r="E122" s="52"/>
       <c r="F122" s="14" t="s">
         <v>266</v>
       </c>
@@ -9038,12 +9038,12 @@
       </c>
     </row>
     <row r="123" spans="1:18" ht="150" customHeight="1">
-      <c r="A123" s="51"/>
-      <c r="B123" s="52"/>
+      <c r="A123" s="52"/>
+      <c r="B123" s="53"/>
       <c r="C123" s="9">
         <v>12</v>
       </c>
-      <c r="D123" s="52"/>
+      <c r="D123" s="53"/>
       <c r="E123" s="10" t="s">
         <v>307</v>
       </c>
@@ -9076,17 +9076,17 @@
       </c>
     </row>
     <row r="124" spans="1:18" ht="150" customHeight="1">
-      <c r="A124" s="51"/>
-      <c r="B124" s="60" t="s">
+      <c r="A124" s="52"/>
+      <c r="B124" s="54" t="s">
         <v>309</v>
       </c>
       <c r="C124" s="9">
         <v>1</v>
       </c>
-      <c r="D124" s="55" t="s">
+      <c r="D124" s="51" t="s">
         <v>310</v>
       </c>
-      <c r="E124" s="55" t="s">
+      <c r="E124" s="51" t="s">
         <v>311</v>
       </c>
       <c r="F124" s="14" t="s">
@@ -9118,13 +9118,13 @@
       </c>
     </row>
     <row r="125" spans="1:18" ht="150" customHeight="1">
-      <c r="A125" s="51"/>
-      <c r="B125" s="51"/>
+      <c r="A125" s="52"/>
+      <c r="B125" s="52"/>
       <c r="C125" s="9">
         <v>2</v>
       </c>
-      <c r="D125" s="51"/>
-      <c r="E125" s="52"/>
+      <c r="D125" s="52"/>
+      <c r="E125" s="53"/>
       <c r="F125" s="14" t="s">
         <v>266</v>
       </c>
@@ -9154,13 +9154,13 @@
       </c>
     </row>
     <row r="126" spans="1:18" ht="150" customHeight="1">
-      <c r="A126" s="51"/>
-      <c r="B126" s="51"/>
+      <c r="A126" s="52"/>
+      <c r="B126" s="52"/>
       <c r="C126" s="9">
         <v>3</v>
       </c>
-      <c r="D126" s="51"/>
-      <c r="E126" s="55" t="s">
+      <c r="D126" s="52"/>
+      <c r="E126" s="51" t="s">
         <v>315</v>
       </c>
       <c r="F126" s="14" t="s">
@@ -9192,13 +9192,13 @@
       </c>
     </row>
     <row r="127" spans="1:18" ht="150" customHeight="1">
-      <c r="A127" s="51"/>
-      <c r="B127" s="51"/>
+      <c r="A127" s="52"/>
+      <c r="B127" s="52"/>
       <c r="C127" s="9">
         <v>4</v>
       </c>
-      <c r="D127" s="51"/>
-      <c r="E127" s="52"/>
+      <c r="D127" s="52"/>
+      <c r="E127" s="53"/>
       <c r="F127" s="14" t="s">
         <v>266</v>
       </c>
@@ -9228,13 +9228,13 @@
       </c>
     </row>
     <row r="128" spans="1:18" ht="150" customHeight="1">
-      <c r="A128" s="51"/>
-      <c r="B128" s="51"/>
+      <c r="A128" s="52"/>
+      <c r="B128" s="52"/>
       <c r="C128" s="9">
         <v>5</v>
       </c>
-      <c r="D128" s="51"/>
-      <c r="E128" s="55" t="s">
+      <c r="D128" s="52"/>
+      <c r="E128" s="51" t="s">
         <v>318</v>
       </c>
       <c r="F128" s="14" t="s">
@@ -9266,13 +9266,13 @@
       </c>
     </row>
     <row r="129" spans="1:18" ht="150" customHeight="1">
-      <c r="A129" s="52"/>
-      <c r="B129" s="52"/>
+      <c r="A129" s="53"/>
+      <c r="B129" s="53"/>
       <c r="C129" s="9">
         <v>6</v>
       </c>
-      <c r="D129" s="52"/>
-      <c r="E129" s="52"/>
+      <c r="D129" s="53"/>
+      <c r="E129" s="53"/>
       <c r="F129" s="14" t="s">
         <v>266</v>
       </c>
@@ -9302,16 +9302,16 @@
       </c>
     </row>
     <row r="130" spans="1:18" ht="150" customHeight="1">
-      <c r="A130" s="55" t="s">
+      <c r="A130" s="51" t="s">
         <v>321</v>
       </c>
-      <c r="B130" s="60" t="s">
+      <c r="B130" s="54" t="s">
         <v>322</v>
       </c>
       <c r="C130" s="9">
         <v>1</v>
       </c>
-      <c r="D130" s="55" t="s">
+      <c r="D130" s="51" t="s">
         <v>323</v>
       </c>
       <c r="E130" s="10" t="s">
@@ -9346,12 +9346,12 @@
       </c>
     </row>
     <row r="131" spans="1:18" ht="150" customHeight="1">
-      <c r="A131" s="51"/>
-      <c r="B131" s="51"/>
+      <c r="A131" s="52"/>
+      <c r="B131" s="52"/>
       <c r="C131" s="9">
         <v>2</v>
       </c>
-      <c r="D131" s="51"/>
+      <c r="D131" s="52"/>
       <c r="E131" s="10" t="s">
         <v>327</v>
       </c>
@@ -9384,13 +9384,13 @@
       </c>
     </row>
     <row r="132" spans="1:18" ht="150" customHeight="1">
-      <c r="A132" s="51"/>
-      <c r="B132" s="51"/>
+      <c r="A132" s="52"/>
+      <c r="B132" s="52"/>
       <c r="C132" s="9">
         <v>3</v>
       </c>
-      <c r="D132" s="51"/>
-      <c r="E132" s="55" t="s">
+      <c r="D132" s="52"/>
+      <c r="E132" s="51" t="s">
         <v>330</v>
       </c>
       <c r="F132" s="14" t="s">
@@ -9420,13 +9420,13 @@
       </c>
     </row>
     <row r="133" spans="1:18" ht="150" customHeight="1">
-      <c r="A133" s="51"/>
-      <c r="B133" s="51"/>
+      <c r="A133" s="52"/>
+      <c r="B133" s="52"/>
       <c r="C133" s="9">
         <v>4</v>
       </c>
-      <c r="D133" s="51"/>
-      <c r="E133" s="52"/>
+      <c r="D133" s="52"/>
+      <c r="E133" s="53"/>
       <c r="F133" s="14" t="s">
         <v>266</v>
       </c>
@@ -9454,13 +9454,13 @@
       </c>
     </row>
     <row r="134" spans="1:18" ht="150" customHeight="1">
-      <c r="A134" s="51"/>
-      <c r="B134" s="51"/>
+      <c r="A134" s="52"/>
+      <c r="B134" s="52"/>
       <c r="C134" s="9">
         <v>5</v>
       </c>
-      <c r="D134" s="51"/>
-      <c r="E134" s="55" t="s">
+      <c r="D134" s="52"/>
+      <c r="E134" s="51" t="s">
         <v>334</v>
       </c>
       <c r="F134" s="14" t="s">
@@ -9490,13 +9490,13 @@
       </c>
     </row>
     <row r="135" spans="1:18" ht="150" customHeight="1">
-      <c r="A135" s="52"/>
-      <c r="B135" s="52"/>
+      <c r="A135" s="53"/>
+      <c r="B135" s="53"/>
       <c r="C135" s="9">
         <v>6</v>
       </c>
-      <c r="D135" s="52"/>
-      <c r="E135" s="52"/>
+      <c r="D135" s="53"/>
+      <c r="E135" s="53"/>
       <c r="F135" s="14" t="s">
         <v>266</v>
       </c>
@@ -9524,16 +9524,16 @@
       </c>
     </row>
     <row r="136" spans="1:18" ht="150" customHeight="1">
-      <c r="A136" s="55" t="s">
+      <c r="A136" s="51" t="s">
         <v>339</v>
       </c>
-      <c r="B136" s="60" t="s">
+      <c r="B136" s="54" t="s">
         <v>340</v>
       </c>
       <c r="C136" s="9">
         <v>1</v>
       </c>
-      <c r="D136" s="55" t="s">
+      <c r="D136" s="51" t="s">
         <v>341</v>
       </c>
       <c r="E136" s="10" t="s">
@@ -9566,12 +9566,12 @@
       </c>
     </row>
     <row r="137" spans="1:18" ht="150" customHeight="1">
-      <c r="A137" s="52"/>
-      <c r="B137" s="52"/>
+      <c r="A137" s="53"/>
+      <c r="B137" s="53"/>
       <c r="C137" s="9">
         <v>2</v>
       </c>
-      <c r="D137" s="52"/>
+      <c r="D137" s="53"/>
       <c r="E137" s="10" t="s">
         <v>345</v>
       </c>
@@ -9602,19 +9602,19 @@
       </c>
     </row>
     <row r="138" spans="1:18" ht="150" customHeight="1">
-      <c r="A138" s="55" t="s">
+      <c r="A138" s="51" t="s">
         <v>349</v>
       </c>
-      <c r="B138" s="60" t="s">
+      <c r="B138" s="54" t="s">
         <v>350</v>
       </c>
       <c r="C138" s="30">
         <v>1</v>
       </c>
-      <c r="D138" s="61" t="s">
+      <c r="D138" s="56" t="s">
         <v>351</v>
       </c>
-      <c r="E138" s="61" t="s">
+      <c r="E138" s="56" t="s">
         <v>352</v>
       </c>
       <c r="F138" s="14" t="s">
@@ -9644,13 +9644,13 @@
       </c>
     </row>
     <row r="139" spans="1:18" ht="150" customHeight="1">
-      <c r="A139" s="51"/>
-      <c r="B139" s="51"/>
+      <c r="A139" s="52"/>
+      <c r="B139" s="52"/>
       <c r="C139" s="30">
         <v>2</v>
       </c>
-      <c r="D139" s="65"/>
-      <c r="E139" s="62"/>
+      <c r="D139" s="57"/>
+      <c r="E139" s="58"/>
       <c r="F139" s="14" t="s">
         <v>266</v>
       </c>
@@ -9678,13 +9678,13 @@
       </c>
     </row>
     <row r="140" spans="1:18" ht="150" customHeight="1">
-      <c r="A140" s="51"/>
-      <c r="B140" s="51"/>
+      <c r="A140" s="52"/>
+      <c r="B140" s="52"/>
       <c r="C140" s="30">
         <v>3</v>
       </c>
-      <c r="D140" s="65"/>
-      <c r="E140" s="61" t="s">
+      <c r="D140" s="57"/>
+      <c r="E140" s="56" t="s">
         <v>356</v>
       </c>
       <c r="F140" s="14" t="s">
@@ -9714,13 +9714,13 @@
       </c>
     </row>
     <row r="141" spans="1:18" ht="150" customHeight="1">
-      <c r="A141" s="51"/>
-      <c r="B141" s="51"/>
+      <c r="A141" s="52"/>
+      <c r="B141" s="52"/>
       <c r="C141" s="30">
         <v>4</v>
       </c>
-      <c r="D141" s="65"/>
-      <c r="E141" s="65"/>
+      <c r="D141" s="57"/>
+      <c r="E141" s="57"/>
       <c r="F141" s="14" t="s">
         <v>266</v>
       </c>
@@ -9748,20 +9748,20 @@
       </c>
     </row>
     <row r="142" spans="1:18" ht="150" customHeight="1">
-      <c r="A142" s="51"/>
-      <c r="B142" s="51"/>
+      <c r="A142" s="52"/>
+      <c r="B142" s="52"/>
       <c r="C142" s="30">
         <v>5</v>
       </c>
-      <c r="D142" s="65"/>
-      <c r="E142" s="65"/>
+      <c r="D142" s="57"/>
+      <c r="E142" s="57"/>
       <c r="F142" s="14" t="s">
         <v>266</v>
       </c>
       <c r="G142" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="H142" s="55" t="s">
+      <c r="H142" s="51" t="s">
         <v>361</v>
       </c>
       <c r="I142" s="10" t="s">
@@ -9782,20 +9782,20 @@
       </c>
     </row>
     <row r="143" spans="1:18" ht="150" customHeight="1">
-      <c r="A143" s="51"/>
-      <c r="B143" s="51"/>
+      <c r="A143" s="52"/>
+      <c r="B143" s="52"/>
       <c r="C143" s="30">
         <v>6</v>
       </c>
-      <c r="D143" s="65"/>
-      <c r="E143" s="62"/>
+      <c r="D143" s="57"/>
+      <c r="E143" s="58"/>
       <c r="F143" s="14" t="s">
         <v>266</v>
       </c>
       <c r="G143" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="H143" s="52"/>
+      <c r="H143" s="53"/>
       <c r="I143" s="10" t="s">
         <v>362</v>
       </c>
@@ -9814,13 +9814,13 @@
       </c>
     </row>
     <row r="144" spans="1:18" ht="150" customHeight="1">
-      <c r="A144" s="51"/>
-      <c r="B144" s="51"/>
+      <c r="A144" s="52"/>
+      <c r="B144" s="52"/>
       <c r="C144" s="30">
         <v>7</v>
       </c>
-      <c r="D144" s="65"/>
-      <c r="E144" s="61" t="s">
+      <c r="D144" s="57"/>
+      <c r="E144" s="56" t="s">
         <v>363</v>
       </c>
       <c r="F144" s="14" t="s">
@@ -9829,10 +9829,10 @@
       <c r="G144" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="H144" s="66" t="s">
+      <c r="H144" s="50" t="s">
         <v>364</v>
       </c>
-      <c r="I144" s="66" t="s">
+      <c r="I144" s="50" t="s">
         <v>365</v>
       </c>
       <c r="J144" s="19" t="s">
@@ -9852,13 +9852,13 @@
       </c>
     </row>
     <row r="145" spans="1:18" ht="150" customHeight="1">
-      <c r="A145" s="51"/>
-      <c r="B145" s="51"/>
+      <c r="A145" s="52"/>
+      <c r="B145" s="52"/>
       <c r="C145" s="30">
         <v>8</v>
       </c>
-      <c r="D145" s="65"/>
-      <c r="E145" s="62"/>
+      <c r="D145" s="57"/>
+      <c r="E145" s="58"/>
       <c r="F145" s="14" t="s">
         <v>266</v>
       </c>
@@ -9886,13 +9886,13 @@
       </c>
     </row>
     <row r="146" spans="1:18" ht="150" customHeight="1">
-      <c r="A146" s="51"/>
-      <c r="B146" s="51"/>
+      <c r="A146" s="52"/>
+      <c r="B146" s="52"/>
       <c r="C146" s="30">
         <v>9</v>
       </c>
-      <c r="D146" s="65"/>
-      <c r="E146" s="63" t="s">
+      <c r="D146" s="57"/>
+      <c r="E146" s="59" t="s">
         <v>368</v>
       </c>
       <c r="F146" s="31" t="s">
@@ -9924,13 +9924,13 @@
       </c>
     </row>
     <row r="147" spans="1:18" ht="150" customHeight="1">
-      <c r="A147" s="51"/>
-      <c r="B147" s="51"/>
+      <c r="A147" s="52"/>
+      <c r="B147" s="52"/>
       <c r="C147" s="30">
         <v>10</v>
       </c>
-      <c r="D147" s="65"/>
-      <c r="E147" s="62"/>
+      <c r="D147" s="57"/>
+      <c r="E147" s="58"/>
       <c r="F147" s="31" t="s">
         <v>266</v>
       </c>
@@ -9958,12 +9958,12 @@
       </c>
     </row>
     <row r="148" spans="1:18" ht="150" customHeight="1">
-      <c r="A148" s="51"/>
-      <c r="B148" s="51"/>
+      <c r="A148" s="52"/>
+      <c r="B148" s="52"/>
       <c r="C148" s="30">
         <v>11</v>
       </c>
-      <c r="D148" s="65"/>
+      <c r="D148" s="57"/>
       <c r="E148" s="33" t="s">
         <v>372</v>
       </c>
@@ -9994,12 +9994,12 @@
       </c>
     </row>
     <row r="149" spans="1:18" ht="150" customHeight="1">
-      <c r="A149" s="51"/>
-      <c r="B149" s="51"/>
+      <c r="A149" s="52"/>
+      <c r="B149" s="52"/>
       <c r="C149" s="30">
         <v>12</v>
       </c>
-      <c r="D149" s="65"/>
+      <c r="D149" s="57"/>
       <c r="E149" s="33" t="s">
         <v>375</v>
       </c>
@@ -10030,13 +10030,13 @@
       </c>
     </row>
     <row r="150" spans="1:18" ht="150" customHeight="1">
-      <c r="A150" s="51"/>
-      <c r="B150" s="51"/>
+      <c r="A150" s="52"/>
+      <c r="B150" s="52"/>
       <c r="C150" s="30">
         <v>13</v>
       </c>
-      <c r="D150" s="65"/>
-      <c r="E150" s="61" t="s">
+      <c r="D150" s="57"/>
+      <c r="E150" s="56" t="s">
         <v>378</v>
       </c>
       <c r="F150" s="14" t="s">
@@ -10066,13 +10066,13 @@
       </c>
     </row>
     <row r="151" spans="1:18" ht="150" customHeight="1">
-      <c r="A151" s="51"/>
-      <c r="B151" s="51"/>
+      <c r="A151" s="52"/>
+      <c r="B151" s="52"/>
       <c r="C151" s="30">
         <v>14</v>
       </c>
-      <c r="D151" s="65"/>
-      <c r="E151" s="62"/>
+      <c r="D151" s="57"/>
+      <c r="E151" s="58"/>
       <c r="F151" s="14" t="s">
         <v>266</v>
       </c>
@@ -10100,13 +10100,13 @@
       </c>
     </row>
     <row r="152" spans="1:18" ht="150" customHeight="1">
-      <c r="A152" s="51"/>
-      <c r="B152" s="51"/>
+      <c r="A152" s="52"/>
+      <c r="B152" s="52"/>
       <c r="C152" s="30">
         <v>15</v>
       </c>
-      <c r="D152" s="65"/>
-      <c r="E152" s="64" t="s">
+      <c r="D152" s="57"/>
+      <c r="E152" s="55" t="s">
         <v>382</v>
       </c>
       <c r="F152" s="34" t="s">
@@ -10138,13 +10138,13 @@
       </c>
     </row>
     <row r="153" spans="1:18" ht="150" customHeight="1">
-      <c r="A153" s="51"/>
-      <c r="B153" s="51"/>
+      <c r="A153" s="52"/>
+      <c r="B153" s="52"/>
       <c r="C153" s="30">
         <v>16</v>
       </c>
-      <c r="D153" s="65"/>
-      <c r="E153" s="51"/>
+      <c r="D153" s="57"/>
+      <c r="E153" s="52"/>
       <c r="F153" s="34" t="s">
         <v>266</v>
       </c>
@@ -10174,12 +10174,12 @@
       </c>
     </row>
     <row r="154" spans="1:18" ht="150" customHeight="1">
-      <c r="A154" s="52"/>
-      <c r="B154" s="52"/>
+      <c r="A154" s="53"/>
+      <c r="B154" s="53"/>
       <c r="C154" s="30">
         <v>17</v>
       </c>
-      <c r="D154" s="62"/>
+      <c r="D154" s="58"/>
       <c r="E154" s="33" t="s">
         <v>387</v>
       </c>
@@ -10212,19 +10212,19 @@
       </c>
     </row>
     <row r="155" spans="1:18" ht="150" customHeight="1">
-      <c r="A155" s="55" t="s">
+      <c r="A155" s="51" t="s">
         <v>390</v>
       </c>
-      <c r="B155" s="60" t="s">
+      <c r="B155" s="54" t="s">
         <v>391</v>
       </c>
       <c r="C155" s="9">
         <v>1</v>
       </c>
-      <c r="D155" s="55" t="s">
+      <c r="D155" s="51" t="s">
         <v>392</v>
       </c>
-      <c r="E155" s="64" t="s">
+      <c r="E155" s="55" t="s">
         <v>393</v>
       </c>
       <c r="F155" s="31" t="s">
@@ -10256,13 +10256,13 @@
       </c>
     </row>
     <row r="156" spans="1:18" ht="150" customHeight="1">
-      <c r="A156" s="51"/>
-      <c r="B156" s="51"/>
+      <c r="A156" s="52"/>
+      <c r="B156" s="52"/>
       <c r="C156" s="9">
         <v>2</v>
       </c>
-      <c r="D156" s="51"/>
-      <c r="E156" s="52"/>
+      <c r="D156" s="52"/>
+      <c r="E156" s="53"/>
       <c r="F156" s="14" t="s">
         <v>266</v>
       </c>
@@ -10292,13 +10292,13 @@
       </c>
     </row>
     <row r="157" spans="1:18" ht="150" customHeight="1">
-      <c r="A157" s="51"/>
-      <c r="B157" s="51"/>
+      <c r="A157" s="52"/>
+      <c r="B157" s="52"/>
       <c r="C157" s="9">
         <v>3</v>
       </c>
-      <c r="D157" s="51"/>
-      <c r="E157" s="55" t="s">
+      <c r="D157" s="52"/>
+      <c r="E157" s="51" t="s">
         <v>398</v>
       </c>
       <c r="F157" s="14" t="s">
@@ -10330,13 +10330,13 @@
       </c>
     </row>
     <row r="158" spans="1:18" ht="150" customHeight="1">
-      <c r="A158" s="52"/>
-      <c r="B158" s="52"/>
+      <c r="A158" s="53"/>
+      <c r="B158" s="53"/>
       <c r="C158" s="9">
         <v>4</v>
       </c>
-      <c r="D158" s="52"/>
-      <c r="E158" s="52"/>
+      <c r="D158" s="53"/>
+      <c r="E158" s="53"/>
       <c r="F158" s="31" t="s">
         <v>266</v>
       </c>
@@ -19630,21 +19630,72 @@
     </row>
   </sheetData>
   <mergeCells count="96">
-    <mergeCell ref="A155:A158"/>
-    <mergeCell ref="B155:B158"/>
-    <mergeCell ref="D155:D158"/>
-    <mergeCell ref="E155:E156"/>
-    <mergeCell ref="E157:E158"/>
-    <mergeCell ref="A138:A154"/>
-    <mergeCell ref="B138:B154"/>
-    <mergeCell ref="D138:D154"/>
-    <mergeCell ref="E138:E139"/>
-    <mergeCell ref="E140:E143"/>
-    <mergeCell ref="H142:H143"/>
-    <mergeCell ref="E144:E145"/>
-    <mergeCell ref="E146:E147"/>
-    <mergeCell ref="E150:E151"/>
-    <mergeCell ref="E152:E153"/>
+    <mergeCell ref="A15:A33"/>
+    <mergeCell ref="B15:B33"/>
+    <mergeCell ref="D15:D33"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="A9:A14"/>
+    <mergeCell ref="B9:B14"/>
+    <mergeCell ref="D9:D11"/>
+    <mergeCell ref="D12:D14"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="H29:H30"/>
+    <mergeCell ref="E15:E17"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="F18:F19"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="E24:E28"/>
+    <mergeCell ref="F24:F28"/>
+    <mergeCell ref="G24:G28"/>
+    <mergeCell ref="A34:A49"/>
+    <mergeCell ref="B34:B49"/>
+    <mergeCell ref="D34:D49"/>
+    <mergeCell ref="A50:A65"/>
+    <mergeCell ref="B50:B65"/>
+    <mergeCell ref="D50:D65"/>
+    <mergeCell ref="A66:A71"/>
+    <mergeCell ref="B66:B71"/>
+    <mergeCell ref="D66:D71"/>
+    <mergeCell ref="A72:A80"/>
+    <mergeCell ref="B72:B80"/>
+    <mergeCell ref="D72:D80"/>
+    <mergeCell ref="E72:E75"/>
+    <mergeCell ref="F72:F73"/>
+    <mergeCell ref="H72:H73"/>
+    <mergeCell ref="A81:A82"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="D81:D82"/>
+    <mergeCell ref="M81:M82"/>
+    <mergeCell ref="A84:A93"/>
+    <mergeCell ref="B84:B93"/>
+    <mergeCell ref="D84:D93"/>
+    <mergeCell ref="E89:E90"/>
+    <mergeCell ref="F89:F90"/>
+    <mergeCell ref="G89:G90"/>
+    <mergeCell ref="A94:A95"/>
+    <mergeCell ref="B94:B95"/>
+    <mergeCell ref="D94:D95"/>
+    <mergeCell ref="A96:A129"/>
+    <mergeCell ref="B96:B103"/>
+    <mergeCell ref="D96:D103"/>
+    <mergeCell ref="B112:B123"/>
+    <mergeCell ref="D112:D123"/>
+    <mergeCell ref="E96:E97"/>
+    <mergeCell ref="E98:E99"/>
+    <mergeCell ref="E100:E101"/>
+    <mergeCell ref="E102:E103"/>
+    <mergeCell ref="B104:B111"/>
+    <mergeCell ref="D104:D111"/>
+    <mergeCell ref="E104:E105"/>
+    <mergeCell ref="E106:E107"/>
+    <mergeCell ref="E108:E109"/>
+    <mergeCell ref="E110:E111"/>
     <mergeCell ref="A136:A137"/>
     <mergeCell ref="B136:B137"/>
     <mergeCell ref="D136:D137"/>
@@ -19660,72 +19711,21 @@
     <mergeCell ref="D130:D135"/>
     <mergeCell ref="E132:E133"/>
     <mergeCell ref="E134:E135"/>
-    <mergeCell ref="E96:E97"/>
-    <mergeCell ref="E98:E99"/>
-    <mergeCell ref="E100:E101"/>
-    <mergeCell ref="E102:E103"/>
-    <mergeCell ref="B104:B111"/>
-    <mergeCell ref="D104:D111"/>
-    <mergeCell ref="E104:E105"/>
-    <mergeCell ref="E106:E107"/>
-    <mergeCell ref="E108:E109"/>
-    <mergeCell ref="E110:E111"/>
-    <mergeCell ref="A94:A95"/>
-    <mergeCell ref="B94:B95"/>
-    <mergeCell ref="D94:D95"/>
-    <mergeCell ref="A96:A129"/>
-    <mergeCell ref="B96:B103"/>
-    <mergeCell ref="D96:D103"/>
-    <mergeCell ref="B112:B123"/>
-    <mergeCell ref="D112:D123"/>
-    <mergeCell ref="M81:M82"/>
-    <mergeCell ref="A84:A93"/>
-    <mergeCell ref="B84:B93"/>
-    <mergeCell ref="D84:D93"/>
-    <mergeCell ref="E89:E90"/>
-    <mergeCell ref="F89:F90"/>
-    <mergeCell ref="G89:G90"/>
-    <mergeCell ref="E72:E75"/>
-    <mergeCell ref="F72:F73"/>
-    <mergeCell ref="H72:H73"/>
-    <mergeCell ref="A81:A82"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="D81:D82"/>
-    <mergeCell ref="A66:A71"/>
-    <mergeCell ref="B66:B71"/>
-    <mergeCell ref="D66:D71"/>
-    <mergeCell ref="A72:A80"/>
-    <mergeCell ref="B72:B80"/>
-    <mergeCell ref="D72:D80"/>
-    <mergeCell ref="A34:A49"/>
-    <mergeCell ref="B34:B49"/>
-    <mergeCell ref="D34:D49"/>
-    <mergeCell ref="A50:A65"/>
-    <mergeCell ref="B50:B65"/>
-    <mergeCell ref="D50:D65"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="G29:G30"/>
-    <mergeCell ref="H29:H30"/>
-    <mergeCell ref="E15:E17"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="F18:F19"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="E24:E28"/>
-    <mergeCell ref="F24:F28"/>
-    <mergeCell ref="G24:G28"/>
-    <mergeCell ref="A15:A33"/>
-    <mergeCell ref="B15:B33"/>
-    <mergeCell ref="D15:D33"/>
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="A9:A14"/>
-    <mergeCell ref="B9:B14"/>
-    <mergeCell ref="D9:D11"/>
-    <mergeCell ref="D12:D14"/>
+    <mergeCell ref="H142:H143"/>
+    <mergeCell ref="E144:E145"/>
+    <mergeCell ref="E146:E147"/>
+    <mergeCell ref="E150:E151"/>
+    <mergeCell ref="E152:E153"/>
+    <mergeCell ref="A138:A154"/>
+    <mergeCell ref="B138:B154"/>
+    <mergeCell ref="D138:D154"/>
+    <mergeCell ref="E138:E139"/>
+    <mergeCell ref="E140:E143"/>
+    <mergeCell ref="A155:A158"/>
+    <mergeCell ref="B155:B158"/>
+    <mergeCell ref="D155:D158"/>
+    <mergeCell ref="E155:E156"/>
+    <mergeCell ref="E157:E158"/>
   </mergeCells>
   <conditionalFormatting sqref="I3">
     <cfRule type="cellIs" dxfId="49" priority="1" stopIfTrue="1" operator="equal">

</xml_diff>

<commit_message>
ok đó, vẫn sai nhưng nhỏ
</commit_message>
<xml_diff>
--- a/CCS.xlsx
+++ b/CCS.xlsx
@@ -2580,7 +2580,7 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
@@ -2604,8 +2604,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="11106150"/>
-          <a:ext cx="3781425" cy="1905000"/>
+          <a:off x="15957176" y="5782235"/>
+          <a:ext cx="3776383" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2617,14 +2617,14 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:colOff>22412</xdr:colOff>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>1904999</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:colOff>22412</xdr:colOff>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>1904999</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2642,8 +2642,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="11106149"/>
-          <a:ext cx="3781425" cy="1905000"/>
+          <a:off x="15979588" y="7687234"/>
+          <a:ext cx="3776383" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2680,7 +2680,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="16821150"/>
+          <a:off x="15944850" y="11496675"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2718,7 +2718,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="18726150"/>
+          <a:off x="15944850" y="13401675"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2732,7 +2732,7 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:row>13</xdr:row>
       <xdr:rowOff>1904999</xdr:rowOff>
     </xdr:from>
     <xdr:to>
@@ -2756,7 +2756,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="53016149"/>
+          <a:off x="15944850" y="17211674"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2770,14 +2770,14 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>1904999</xdr:rowOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>1904999</xdr:rowOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2794,8 +2794,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="54921149"/>
-          <a:ext cx="3781425" cy="1905000"/>
+          <a:off x="15957176" y="19117235"/>
+          <a:ext cx="3776383" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2832,7 +2832,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="56826150"/>
+          <a:off x="15944850" y="21021675"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2846,14 +2846,14 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>140</xdr:row>
-      <xdr:rowOff>1904999</xdr:rowOff>
+      <xdr:row>141</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>141</xdr:row>
-      <xdr:rowOff>1904999</xdr:rowOff>
+      <xdr:row>142</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2870,7 +2870,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="264471149"/>
+          <a:off x="15944850" y="59121675"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2908,7 +2908,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="266376150"/>
+          <a:off x="15944850" y="61026675"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2946,8 +2946,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15957176" y="268280029"/>
-          <a:ext cx="3776383" cy="1905000"/>
+          <a:off x="15944850" y="62931675"/>
+          <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2984,7 +2984,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="279711150"/>
+          <a:off x="15944850" y="72456675"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2998,14 +2998,14 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>143</xdr:row>
-      <xdr:rowOff>1904999</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>144</xdr:row>
-      <xdr:rowOff>1904999</xdr:rowOff>
+      <xdr:row>145</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3022,7 +3022,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="270186149"/>
+          <a:off x="15944850" y="64836675"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3036,7 +3036,7 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>145</xdr:row>
+      <xdr:row>144</xdr:row>
       <xdr:rowOff>1904999</xdr:rowOff>
     </xdr:from>
     <xdr:to>
@@ -3060,7 +3060,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="273996149"/>
+          <a:off x="15944850" y="66741674"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3074,7 +3074,7 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>80</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
@@ -3098,7 +3098,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="148266150"/>
+          <a:off x="15944850" y="22926675"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3136,7 +3136,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="150171150"/>
+          <a:off x="15944850" y="24831675"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3150,14 +3150,14 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>82</xdr:row>
-      <xdr:rowOff>1904999</xdr:rowOff>
+      <xdr:row>83</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>83</xdr:row>
-      <xdr:rowOff>1904999</xdr:rowOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3174,7 +3174,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="153981149"/>
+          <a:off x="15944850" y="28641675"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3212,7 +3212,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="155886150"/>
+          <a:off x="15944850" y="30546675"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3250,7 +3250,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="157791150"/>
+          <a:off x="15944850" y="32451675"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3288,7 +3288,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="159696150"/>
+          <a:off x="15944850" y="34356675"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3302,7 +3302,7 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>90</xdr:row>
+      <xdr:row>87</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
@@ -3326,7 +3326,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="167316150"/>
+          <a:off x="15944850" y="36261675"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3340,14 +3340,14 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>90</xdr:row>
-      <xdr:rowOff>1904999</xdr:rowOff>
+      <xdr:row>91</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>91</xdr:row>
-      <xdr:rowOff>1904999</xdr:rowOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3364,7 +3364,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15944850" y="169221149"/>
+          <a:off x="15944850" y="38166675"/>
           <a:ext cx="3781425" cy="1905000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">

</xml_diff>